<commit_message>
Separar los dos oficios: pintor y ebanista
- Página: secciones El pintor y El ebanista, y bloque de catálogos y hojas de vida
- Catálogo de arte (7 págs.) y catálogo de ebanistería (6 págs.) con código común
- Hoja de vida artística y hoja de vida como ebanista sobre una plantilla común
- datos.js: PERFIL.arte / PERFIL.madera, SERVICIOS y campo area en la trayectoria
- Plantilla de Excel con columna area; README actualizado

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xg453ancghpBkrbYp1DerW
</commit_message>
<xml_diff>
--- a/contenido/contenido-pagina-santamaria.xlsx
+++ b/contenido/contenido-pagina-santamaria.xlsx
@@ -448,7 +448,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Cómo actualizar la página, el catálogo y la hoja de vida desde esta hoja</t>
+          <t>Cómo actualizar la página, los catálogos y las hojas de vida desde esta hoja</t>
         </is>
       </c>
     </row>
@@ -475,21 +475,21 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Pestaña obras (galería de la página y colección del catálogo)</t>
+          <t>Pestaña obras</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  categoria: pintura, dibujo o ebanisteria (lista desplegable).</t>
+          <t xml:space="preserve">  categoria: pintura o dibujo → sección y catálogo del pintor; ebanisteria → sección y catálogo del ebanista.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  imagen: ruta dentro del sitio (img/obras/archivo.jpg) o enlace de Google Drive compartido como "Cualquier persona con el enlace". Vacío = marcador "Fotografía próximamente".</t>
+          <t xml:space="preserve">  imagen: ruta dentro del sitio (img/obras/archivo.jpg) o enlace de Google Drive compartido como "Cualquier persona con el enlace". Vacío = "Fotografía próximamente".</t>
         </is>
       </c>
     </row>
@@ -503,24 +503,24 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  destacada: si → la obra aparece en el catálogo, 4 por página.</t>
+          <t xml:space="preserve">  destacada: si → la obra aparece en el catálogo de arte, 4 por página.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Técnica y medidas vacías o marcadas deben confirmarse con el maestro.</t>
-        </is>
-      </c>
+      <c r="A11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Pestaña trayectoria</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Pestaña trayectoria (línea de tiempo, página de trayectoria del catálogo y hoja de vida)</t>
+          <t xml:space="preserve">  area: arte (pintor), madera (ebanista) o ambas. Decide en qué hoja de vida y en qué sección de la página aparece.</t>
         </is>
       </c>
     </row>
@@ -1324,44 +1324,50 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="34" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
           <t>anio</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>tipo</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>titulo</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>lugar</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>detalle</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>certificado</t>
         </is>
@@ -1370,994 +1376,1256 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
+          <t>arte</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
           <t>Desde niño</t>
         </is>
       </c>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>formacion</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>Formación empírica en pintura, talla y carpintería</t>
-        </is>
-      </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
+          <t>Formación empírica en pintura</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
           <t>San Martín de los Llanos, Meta</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>Pintaba paisajes y personajes de su región, moldeaba arcilla y tallaba madera. Aprendió la carpintería en el entorno familiar.</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr"/>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>En sus cuadernos de escuela degradaba colores y sombras para pintar los paisajes y personajes de su región, y moldeaba arcilla.</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>1990 – 2002</t>
+          <t>madera</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>experiencia</t>
+          <t>Desde niño</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>Pintor independiente</t>
+          <t>formacion</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>Bogotá</t>
+          <t>Formación empírica en carpintería y talla</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>Doce años de trabajo pictórico continuo, abriéndose camino con coleccionistas y clientes de arte en la capital.</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr"/>
+          <t>San Martín de los Llanos, Meta</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Aprendió el oficio en el taller familiar de carpintería y tallaba madera desde la escuela.</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>2002 – 2015</t>
+          <t>arte</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
+          <t>1990 – 2002</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
           <t>experiencia</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Fundador de una fábrica de muebles</t>
-        </is>
-      </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Meta, Colombia</t>
+          <t>Pintor independiente</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Durante trece años su empresa surtió de muebles al departamento del Meta.</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr"/>
+          <t>Bogotá</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Doce años de trabajo pictórico continuo, abriéndose camino con coleccionistas y clientes de arte en la capital.</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2016 – 2021</t>
+          <t>madera</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
+          <t>2002 – 2015</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
           <t>experiencia</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Artista plástico en Nueva York y Nueva Jersey</t>
-        </is>
-      </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>Fundador y director de una fábrica de muebles</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Exposiciones colectivas con el New Jersey Artist Collective, consulados y organizaciones culturales latinas; retratos y obra por encargo.</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr"/>
+          <t>San Martín de los Llanos, Meta</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Diseño, fabricación y venta de muebles. Durante trece años su empresa surtió al departamento del Meta.</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Actualidad</t>
+          <t>arte</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
+          <t>2016 – 2021</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
           <t>experiencia</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Taller de pintura y ebanistería</t>
-        </is>
-      </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Meta, Colombia</t>
+          <t>Artista plástico en Nueva York y Nueva Jersey</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Obra original, retratos por encargo, marcos, bastidores, muebles y puertas a medida, y talleres de formación.</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr"/>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Exposiciones colectivas con el New Jersey Artist Collective, consulados y organizaciones culturales latinas; retratos y obra por encargo.</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>arte</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>exposicion</t>
+          <t>Actualidad</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Cartas de Amor y Arte</t>
+          <t>experiencia</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Bethune Center, Jersey City, NJ · 20 de abril</t>
+          <t>Taller de pintura</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Exposición de arte y literatura del New Jersey Artist Collective, La Magia de las Bellas Artes y la Fundación El Sol Sale para Todos.</t>
+          <t>Meta, Colombia</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-15.jpg</t>
-        </is>
-      </c>
+          <t>Obra original, retratos por encargo y talleres de pintura y dibujo.</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>madera</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>exposicion</t>
+          <t>Actualidad</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Ecléctica</t>
+          <t>experiencia</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>Mason Civic League, Hoboken, NJ · 7 al 20 de julio</t>
+          <t>Taller de ebanistería y carpintería</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Muestra colectiva curada por Amado Mora y Juan Ramiro Torres.</t>
+          <t>Meta, Colombia</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-17.jpg,img/certificados/cert-05.jpg</t>
-        </is>
-      </c>
+          <t>Muebles, puertas, closets y cocinas a la medida; marcos de autor, bastidores y restauración.</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>madera</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>exposicion</t>
+          <t>Desde sus inicios</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Muestra de Arte en Rosado</t>
+          <t>experiencia</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>Elizabeth, NJ · 13 de julio</t>
+          <t>Marcos y bastidores para su propia obra</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Organizada por el Consulado de El Salvador para Nueva Jersey y Delaware y el New Jersey Artist Collective, por el Día de la Prevención contra el Cáncer.</t>
+          <t>Colombia y Estados Unidos</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-02.jpg</t>
-        </is>
-      </c>
+          <t>Construye los soportes y marcos de sus pinturas, uniendo los dos oficios en cada pieza.</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
+          <t>arte</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
           <t>2018</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>exposicion</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>Huellas Trashumantes · Exhibición Internacional de Arte</t>
-        </is>
-      </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>Nueva York · 18 al 24 de julio</t>
+          <t>Cartas de Amor y Arte</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Organizada por Arte al Paso Gallery con el apoyo del New Jersey Artist Collective y el Comisionado Dominicano de Cultura.</t>
+          <t>Bethune Center, Jersey City, NJ · 20 de abril</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-18.jpg</t>
+          <t>Exposición de arte y literatura del New Jersey Artist Collective, La Magia de las Bellas Artes y la Fundación El Sol Sale para Todos.</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-15.jpg</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
+          <t>arte</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
           <t>2018</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>exposicion</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>Celebración de la Herencia Hispana</t>
-        </is>
-      </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>Union County Performing Arts Center, Rahway, NJ · 23 de septiembre</t>
+          <t>Ecléctica</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Certificado de participación de la Junta de Freeholders del Condado de Union.</t>
+          <t>Mason Civic League, Hoboken, NJ · 7 al 20 de julio</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-01.jpg</t>
+          <t>Muestra colectiva curada por Amado Mora y Juan Ramiro Torres.</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-17.jpg,img/certificados/cert-05.jpg</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
+          <t>arte</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
           <t>2018</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="C12" s="4" t="inlineStr">
         <is>
           <t>exposicion</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Black &amp; White</t>
-        </is>
-      </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>AC-PIX Studio, Union City, NJ · 14 de diciembre</t>
+          <t>Muestra de Arte en Rosado</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Su obra en carbón fue la imagen del afiche de la exposición.</t>
+          <t>Elizabeth, NJ · 13 de julio</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-04.jpg,img/certificados/cert-03.jpg</t>
+          <t>Organizada por el Consulado de El Salvador para Nueva Jersey y Delaware y el New Jersey Artist Collective, por el Día de la Prevención contra el Cáncer.</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-02.jpg</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>arte</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
           <t>exposicion</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Muestra de Arte en Rosado</t>
-        </is>
-      </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Queens, NY · 16 de febrero</t>
+          <t>Huellas Trashumantes · Exhibición Internacional de Arte</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>Mujeres Exitosas NY, por el Día de la Prevención contra el Cáncer.</t>
+          <t>Nueva York · 18 al 24 de julio</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-26.jpg</t>
+          <t>Organizada por Arte al Paso Gallery con el apoyo del New Jersey Artist Collective y el Comisionado Dominicano de Cultura.</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-18.jpg</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>arte</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
           <t>exposicion</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Día Internacional del Niño</t>
-        </is>
-      </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Nueva York · 6 de abril</t>
+          <t>Celebración de la Herencia Hispana</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Diploma de agradecimiento del Comité Cívico Cultural Boliviano de Nueva York.</t>
+          <t>Union County Performing Arts Center, Rahway, NJ · 23 de septiembre</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-27.jpg</t>
+          <t>Certificado de participación de la Junta de Freeholders del Condado de Union.</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-01.jpg</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>arte</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
           <t>exposicion</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Celebrating International Day for the Children</t>
-        </is>
-      </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>The Latin American Institute · 28 de abril</t>
+          <t>Black &amp; White</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>Muestra de pintura, dibujo, escultura y fotografía curada por Amado Mora.</t>
+          <t>AC-PIX Studio, Union City, NJ · 14 de diciembre</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-06.jpg</t>
+          <t>Su obra en carbón fue la imagen del afiche de la exposición.</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-04.jpg,img/certificados/cert-03.jpg</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
+          <t>arte</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="C16" s="4" t="inlineStr">
         <is>
           <t>exposicion</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Exposición del Día de la Madre</t>
-        </is>
-      </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Consulado del Ecuador en Queens, NY · 4 de mayo</t>
+          <t>Muestra de Arte en Rosado</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Certificado de agradecimiento por su aporte cultural a la comunidad migrante.</t>
+          <t>Queens, NY · 16 de febrero</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-25.jpg</t>
+          <t>Mujeres Exitosas NY, por el Día de la Prevención contra el Cáncer.</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-26.jpg</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
+          <t>arte</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="C17" s="4" t="inlineStr">
         <is>
           <t>exposicion</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Mujeres en el Poder</t>
-        </is>
-      </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Manhattan, NY · 20 al 24 de agosto</t>
+          <t>Día Internacional del Niño</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>Exhibición colectiva de la Asamblea Nacional del Ecuador en celebración de las mujeres que inspiran.</t>
+          <t>Nueva York · 6 de abril</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-29.jpg</t>
+          <t>Diploma de agradecimiento del Comité Cívico Cultural Boliviano de Nueva York.</t>
+        </is>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-27.jpg</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
+          <t>arte</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="C18" s="4" t="inlineStr">
         <is>
           <t>exposicion</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>VIVA Bradley Beach!</t>
-        </is>
-      </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Bradley Beach, NJ · 14 de septiembre</t>
+          <t>Celebrating International Day for the Children</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Certificado de participación de la Comisión de Turismo de Bradley Beach.</t>
+          <t>The Latin American Institute · 28 de abril</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-14.jpg</t>
+          <t>Muestra de pintura, dibujo, escultura y fotografía curada por Amado Mora.</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-06.jpg</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
+          <t>arte</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="C19" s="4" t="inlineStr">
         <is>
           <t>exposicion</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>Arte en Rosado 2019</t>
-        </is>
-      </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Nueva Jersey</t>
+          <t>Exposición del Día de la Madre</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Asociación Iberoamericana Unida USA, New Jersey Artist Collective, They Have a Name y F.A.I.T.H.</t>
+          <t>Consulado del Ecuador en Queens, NY · 4 de mayo</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-13.jpg</t>
+          <t>Certificado de agradecimiento por su aporte cultural a la comunidad migrante.</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-25.jpg</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
+          <t>arte</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="C20" s="4" t="inlineStr">
         <is>
           <t>exposicion</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>Black and White Art Expo</t>
-        </is>
-      </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>Hoboken, NJ · 29 de noviembre</t>
+          <t>Mujeres en el Poder</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>New Jersey Artist Collective, They Have a Name y F.A.I.T.H.</t>
+          <t>Manhattan, NY · 20 al 24 de agosto</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-11.jpg</t>
+          <t>Exhibición colectiva de la Asamblea Nacional del Ecuador en celebración de las mujeres que inspiran.</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-29.jpg</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
+          <t>arte</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>exposicion</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>To Sir, With Love Art Exp. 2019</t>
-        </is>
-      </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Garfield, NJ · 30 de noviembre</t>
+          <t>VIVA Bradley Beach!</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Reconocimiento especial del Colectivo de Artistas de New Jersey.</t>
+          <t>Bradley Beach, NJ · 14 de septiembre</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-10.jpg</t>
+          <t>Certificado de participación de la Comisión de Turismo de Bradley Beach.</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-14.jpg</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>arte</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
           <t>exposicion</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>Earth Day Art Expo 2021</t>
-        </is>
-      </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Second Ave. Firehouse Gallery, Bay Shore, NY · 24 de abril</t>
+          <t>Arte en Rosado 2019</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Certificado de reconocimiento del Teatro Experimental Yerbabruja.</t>
+          <t>Nueva Jersey</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-09.jpg</t>
+          <t>Asociación Iberoamericana Unida USA, New Jersey Artist Collective, They Have a Name y F.A.I.T.H.</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-13.jpg</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>2021</t>
+          <t>arte</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
           <t>exposicion</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>Ever Green Art Expo 2021 · Artista destacado</t>
-        </is>
-      </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>PRONTO of Long Island, NY</t>
+          <t>Black and White Art Expo</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Artista invitado del Lobby Art Show.</t>
+          <t>Hoboken, NJ · 29 de noviembre</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-08.jpg</t>
+          <t>New Jersey Artist Collective, They Have a Name y F.A.I.T.H.</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-11.jpg</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr"/>
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>arte</t>
+        </is>
+      </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
           <t>exposicion</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>Arte Joven · Colombia Fest</t>
-        </is>
-      </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>V Feria de Servicios</t>
+          <t>To Sir, With Love Art Exp. 2019</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Participó con la obra "Solidaridad y bondad", óleo sobre lienzo de 36 × 48 pulgadas.</t>
+          <t>Garfield, NJ · 30 de noviembre</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-23.jpg</t>
+          <t>Reconocimiento especial del Colectivo de Artistas de New Jersey.</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-10.jpg</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>arte</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>reconocimiento</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Premios Talentos Latinos 2018 de Colombia</t>
+          <t>exposicion</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Ciudad Latina FM</t>
+          <t>Earth Day Art Expo 2021</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Reconocimiento a la obra "Shakira".</t>
+          <t>Second Ave. Firehouse Gallery, Bay Shore, NY · 24 de abril</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-20.jpg</t>
+          <t>Certificado de reconocimiento del Teatro Experimental Yerbabruja.</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-09.jpg</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>2018</t>
+          <t>arte</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>reconocimiento</t>
+          <t>2021</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Premios Latinos del Mundo New York VIP 2018</t>
+          <t>exposicion</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>Nueva York</t>
+          <t>Ever Green Art Expo 2021 · Artista destacado</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Reconocimiento al Talento Colombiano, otorgado por Anafiestas Entertainment.</t>
+          <t>PRONTO of Long Island, NY</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-21.jpg,img/certificados/cert-22.jpg</t>
+          <t>Artista invitado del Lobby Art Show.</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-08.jpg</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>2018</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>reconocimiento</t>
-        </is>
-      </c>
+          <t>arte</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr"/>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Latino NY Awards</t>
+          <t>exposicion</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Nueva York</t>
+          <t>Arte Joven · Colombia Fest</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>Reconocimiento "Artista en el Arte", Orgullo Hispano 2018.</t>
+          <t>V Feria de Servicios</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-24.jpg</t>
+          <t>Participó con la obra "Solidaridad y bondad", óleo sobre lienzo de 36 × 48 pulgadas.</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-23.jpg</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
+          <t>arte</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
           <t>2018</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>reconocimiento</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>Asamblea Nacional del Ecuador</t>
-        </is>
-      </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Centro de Arte Julia de Burgos, Nueva York · 5 de septiembre</t>
+          <t>Premios Talentos Latinos 2018 de Colombia</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Reconocimiento al artista por su participación en la exhibición colectiva "Mujer: Inmigración y Progreso".</t>
+          <t>Ciudad Latina FM</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-19.jpg</t>
+          <t>Reconocimiento a la obra "Shakira".</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-20.jpg</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>arte</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
           <t>reconocimiento</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>The Latin American Institute</t>
-        </is>
-      </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>Hackensack, NJ · 3 de mayo</t>
+          <t>Premios Latinos del Mundo New York VIP 2018</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>Reconocimiento especial, con la curaduría de Amado Mora.</t>
+          <t>Nueva York</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-07.jpg</t>
+          <t>Reconocimiento al Talento Colombiano, otorgado por Anafiestas Entertainment.</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-21.jpg,img/certificados/cert-22.jpg</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>arte</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
           <t>reconocimiento</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>Certificado de apreciación</t>
-        </is>
-      </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Nueva Jersey · 11 de noviembre</t>
+          <t>Latino NY Awards</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>Por sus contribuciones a Clear Choices, New Jersey Artist Collective, They Have a Name, F.A.I.T.H. y Latin Project Foundations.</t>
+          <t>Nueva York</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-12.jpg</t>
+          <t>Reconocimiento "Artista en el Arte", Orgullo Hispano 2018.</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-24.jpg</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr"/>
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>arte</t>
+        </is>
+      </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
           <t>reconocimiento</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>Consulado del Ecuador en Queens</t>
-        </is>
-      </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>Nueva York</t>
+          <t>Asamblea Nacional del Ecuador</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>Reconocimiento por su destacada trayectoria y desempeño artístico, enalteciendo la cultura en el exterior.</t>
+          <t>Centro de Arte Julia de Burgos, Nueva York · 5 de septiembre</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
         <is>
-          <t>img/certificados/cert-16.jpg</t>
+          <t>Reconocimiento al artista por su participación en la exhibición colectiva "Mujer: Inmigración y Progreso".</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-19.jpg</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>2024</t>
+          <t>arte</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>hito</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Retrato por encargo en carbón y pastel</t>
+          <t>reconocimiento</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>Estados Unidos</t>
+          <t>The Latin American Institute</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>Pieza de gran formato, 91 × 122 cm, entregada personalmente a su destinataria.</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr"/>
+          <t>Hackensack, NJ · 3 de mayo</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Reconocimiento especial, con la curaduría de Amado Mora.</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-07.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
+          <t>arte</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>reconocimiento</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Certificado de apreciación</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Nueva Jersey · 11 de noviembre</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Por sus contribuciones a Clear Choices, New Jersey Artist Collective, They Have a Name, F.A.I.T.H. y Latin Project Foundations.</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-12.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>arte</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr"/>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>reconocimiento</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>Consulado del Ecuador en Queens</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Nueva York</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Reconocimiento por su destacada trayectoria y desempeño artístico, enalteciendo la cultura en el exterior.</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>img/certificados/cert-16.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>arte</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>hito</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>Retrato por encargo en carbón y pastel</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Estados Unidos</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>Pieza de gran formato, 91 × 122 cm, entregada personalmente a su destinataria.</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>ambas</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
           <t>Actualidad</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>hito</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr">
         <is>
           <t>Regreso al Meta</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="E36" s="4" t="inlineStr">
         <is>
           <t>Meta, Colombia</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="F36" s="4" t="inlineStr">
         <is>
           <t>Pintura, ebanistería de autor y formación comunitaria desde su tierra natal.</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr"/>
+      <c r="G36" s="4" t="inlineStr"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="B2:B300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+  <dataValidations count="2">
+    <dataValidation sqref="A2:A300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"arte,madera,ambas"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"experiencia,exposicion,reconocimiento,formacion,hito"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>